<commit_message>
Add new Excel configuration files for item and role settings
- Created '物品配置.xlsx' for item configurations with 5225 rows.
- Created '角色配置.xlsx' for role configurations with 5327 rows.
</commit_message>
<xml_diff>
--- a/test/test_output/realistic_test_result.xlsx
+++ b/test/test_output/realistic_test_result.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,26 +27,15 @@
     </font>
     <font>
       <b val="1"/>
-      <sz val="12"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFC000"/>
-        <bgColor rgb="00FFC000"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -73,12 +62,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -450,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -460,57 +446,48 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1">
-        <f>== 有文本内容的表格 ===</f>
-        <v/>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>表名</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>工作表</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>字段数量</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>字段+示例</t>
+        </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>表名</t>
+          <t>game_config_realistic.xlsx</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>工作表</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>字段数量</t>
-        </is>
+          <t>关卡配置</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>4</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>字段+示例</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>game_config_realistic.xlsx</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>关卡配置</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>level_name,新手村, level_desc,这是新手村的关卡，难度简单, difficulty,简单, reward_desc,获得100金币和经验</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>